<commit_message>
refactor: Item.IconPath 改名 SpriteId（存的是逻辑图ID不是路径）
语义更准确：SpriteId 指向 UISprite 表的 Id（如 icon_sword），
业务 GetSpriteById(item.SpriteId) 取图。生成物已随导出更新。
</commit_message>
<xml_diff>
--- a/Assets/Config/Excel/Item.xlsx
+++ b/Assets/Config/Excel/Item.xlsx
@@ -474,7 +474,7 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>IconPath</t>
+          <t>SpriteId</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
@@ -675,7 +675,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>图标(只客户端)</t>
+          <t>图ID(填 UISprite 表的 Id)</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">

</xml_diff>